<commit_message>
Fix #32216 - [Bug] Remove hidden excel sheet in labelClaimList spec export
</commit_message>
<xml_diff>
--- a/becpg-plm/becpg-plm-core/src/main/resources/beCPG/birt/exportsearch/spec/fr/ExportSpecLabelClaimList.xlsx
+++ b/becpg-plm/becpg-plm-core/src/main/resources/beCPG/birt/exportsearch/spec/fr/ExportSpecLabelClaimList.xlsx
@@ -5,16 +5,15 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="1" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Produits" sheetId="1" state="hidden" r:id="rId2"/>
-    <sheet name="Produit" sheetId="2" state="visible" r:id="rId3"/>
-    <sheet name="Allégations" sheetId="3" state="visible" r:id="rId4"/>
+    <sheet name="Produit" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Allégations" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Allégations!$A$3:$L$3</definedName>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Produit!$A$3:$H$3</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Allégations!$A$3:$L$3</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Produit!$A$3:$H$3</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -26,66 +25,48 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="38">
   <si>
     <t xml:space="preserve">TYPE</t>
   </si>
   <si>
-    <t xml:space="preserve">bcpg:finishedProduct</t>
+    <t xml:space="preserve">bcpg:productSpecification</t>
   </si>
   <si>
     <t xml:space="preserve">COLUMNS</t>
   </si>
   <si>
+    <t xml:space="preserve">cm:name</t>
+  </si>
+  <si>
     <t xml:space="preserve">bcpg:code</t>
   </si>
   <si>
     <t xml:space="preserve">bcpg:erpCode</t>
   </si>
   <si>
-    <t xml:space="preserve">cm:name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dyn_Taux_de_gâche_(%)_SF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dyn_Productivité__SF</t>
+    <t xml:space="preserve">bcpg:productHierarchy1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bcpg:productHierarchy2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cm:description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bcpg:legalName</t>
   </si>
   <si>
     <t xml:space="preserve">#</t>
   </si>
   <si>
-    <t xml:space="preserve">Code produit</t>
+    <t xml:space="preserve">Nom</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Code beCPG</t>
   </si>
   <si>
     <t xml:space="preserve">Code ERP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nom</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Taux de gâche SF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Productivité SF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bcpg:productSpecification</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bcpg:productHierarchy1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bcpg:productHierarchy2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cm:description</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bcpg:legalName</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Code beCPG</t>
   </si>
   <si>
     <t xml:space="preserve">Famille</t>
@@ -167,7 +148,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -189,14 +170,6 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
@@ -222,7 +195,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -231,30 +204,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFBDD7EE"/>
-        <bgColor rgb="FF99CCFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FF004254"/>
         <bgColor rgb="FF003300"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
       <diagonal/>
     </border>
   </borders>
@@ -288,27 +248,27 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -325,15 +285,15 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00FFFFFF"/>
+          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFF7F7F7"/>
-          <bgColor rgb="FF272727"/>
+          <fgColor rgb="FF000000"/>
+          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -341,6 +301,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF004254"/>
+          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -348,6 +309,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -377,7 +339,7 @@
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFBDD7EE"/>
+      <rgbColor rgb="FFCCCCFF"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -423,157 +385,188 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="8.55859375" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="1" min="1" style="0" width="9.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13.55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="26.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="20.33"/>
-  </cols>
-  <sheetData>
-    <row r="1" customFormat="false" ht="14.4" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="0" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="14.4" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="0" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="E2" s="0" t="s">
-        <v>6</v>
-      </c>
-      <c r="F2" s="0" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="0" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" s="0" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12Page &amp;P</oddFooter>
-  </headerFooter>
-</worksheet>
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+  <a:themeElements>
+    <a:clrScheme name="LibreOffice">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="ffffff"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="000000"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="ffffff"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="18a303"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="0369a3"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="a33e03"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8e03a3"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="c99c00"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="c9211e"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000ee"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="551a8b"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme>
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultColWidth="11.45703125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.4609375" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="1" min="1" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.69"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13.78"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="20.62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="41.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="35.62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1024" style="0" width="9.14"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="1" min="1" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="25.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="13.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="20.62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="41.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="35.62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1024" style="1" width="9.14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
-        <v>14</v>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="0" t="s">
-        <v>3</v>
-      </c>
-      <c r="D2" s="0" t="s">
-        <v>4</v>
-      </c>
-      <c r="E2" s="0" t="s">
+      <c r="E2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" s="2" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="G3" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="0" t="s">
+      <c r="H3" s="3" t="s">
         <v>17</v>
-      </c>
-      <c r="H2" s="0" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="3" s="3" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -589,109 +582,109 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L3"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="1" min="1" style="0" width="16.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="17.64"/>
-    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="3" min="3" style="0" width="42.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="0" width="40.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="19.85"/>
-    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="8" min="8" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="24.64"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="26.21"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="30.09"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="19.89"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="1" min="1" style="1" width="16.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17.64"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="3" min="3" style="1" width="42.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="1" width="40.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="19.85"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="8" min="8" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="24.64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="26.21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="30.09"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="19.89"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
+      <c r="B1" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="H2" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="L2" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="G2" s="0" t="s">
+    </row>
+    <row r="3" s="2" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="H2" s="0" t="s">
+      <c r="F3" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="I2" s="0" t="s">
+      <c r="G3" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="J2" s="0" t="s">
+      <c r="H3" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="K2" s="0" t="s">
+      <c r="I3" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="L2" s="0" t="s">
+      <c r="J3" s="3" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="3" s="3" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" s="4" t="s">
+      <c r="K3" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="L3" s="3" t="s">
         <v>37</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="H3" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="J3" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="K3" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="L3" s="4" t="s">
-        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>